<commit_message>
Add all lessons for database automation on PostgreSQL
The plan now runs theory before the matching practice and uses PostgreSQL 16 in the training Linux VM instead of SQLite. All 29 lessons are written: 17 lectures with three gates and 15-question tests, 12 practices with the seven-section template, evidence screenshots and self-check questions without answers. The discipline is available, all lessons are open, and the Excel plan totals 66 hours.
</commit_message>
<xml_diff>
--- a/courses/4/db-automation/dist/Учебный_план_Управление_и_автоматизация_баз_данных.xlsx
+++ b/courses/4/db-automation/dist/Учебный_план_Управление_и_автоматизация_баз_данных.xlsx
@@ -212,12 +212,12 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 1. Установка SQLite/клиент</t>
+          <t xml:space="preserve">Лекция 2. Архитектура PostgreSQL</t>
         </is>
       </c>
       <c r="D7" s="6">
@@ -225,16 +225,16 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты устанавливают SQLite и клиент, создают учебную базу и подключаются к ней из командной строки. Сдают файл базы и протокол проверки подключения.</t>
+          <t xml:space="preserve">PostgreSQL делится на процессы, разделяемую память и файлы WAL; от этой раскладки зависит поведение запросов. Разбираются клиент-серверная и файловая модели.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">файл базы, подключение, командная строка, версия, порт</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="45" customHeight="1">
+          <t xml:space="preserve">ядро, клиент-сервер, буферный кэш, журнал, файл данных, процесс</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="60" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">3</t>
@@ -247,7 +247,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 2. Архитектура СУБД</t>
+          <t xml:space="preserve">Лекция 3. Установка и настройка PostgreSQL</t>
         </is>
       </c>
       <c r="D8" s="6">
@@ -255,12 +255,12 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">СУБД делится на процессы, память и файлы на диске, и от этой раскладки зависит поведение запросов. Разбираются клиент-серверная и файловая модели.</t>
+          <t xml:space="preserve">Настройка PostgreSQL сводится к расположению файлов, памяти, WAL и сетевому доступу. Разбирается, что менять и как проверить результат после перезапуска.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ядро, клиент-сервер, буферный кэш, журнал, файл данных, процесс</t>
+          <t xml:space="preserve">конфигурация, параметр, кэш, журнал, порт, перезапуск</t>
         </is>
       </c>
     </row>
@@ -277,117 +277,117 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Практика 1. Установка PostgreSQL и подключение</t>
+        </is>
+      </c>
+      <c r="D9" s="6">
+        <v>2</v>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Студенты устанавливают PostgreSQL в учебной Linux VM, создают учебную базу и подключаются к ней через psql. Сдают протокол установки, список баз и проверку подключения.</t>
+        </is>
+      </c>
+      <c r="F9" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">PostgreSQL, VirtualBox, psql, createdb, подключение, порт 5432</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 4. Пользователи и роли</t>
+        </is>
+      </c>
+      <c r="D10" s="6">
+        <v>2</v>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Доступ к данным строится на ролях, а не на отдельных аккаунтах. Разбираются привилегии, владение объектами и проверка выданных прав.</t>
+        </is>
+      </c>
+      <c r="F10" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">привилегия, владелец объекта, схема, GRANT, аудит прав, наследование ролей</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="60" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C11" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Практика 2. Пользователи и роли</t>
         </is>
       </c>
-      <c r="D9" s="6">
-        <v>2</v>
-      </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="D11" s="6">
+        <v>2</v>
+      </c>
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Студенты создают пользователей учебной базы, выдают права через роли и проверяют доступ от каждого аккаунта. Сдают SQL-скрипт с ролями и таблицу проверки прав.</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">привилегия, GRANT, REVOKE, минимальные привилегии, учётная запись, проверка доступа</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="60" customHeight="1">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">5</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 3. Установка и настройка</t>
-        </is>
-      </c>
-      <c r="D10" s="6">
-        <v>2</v>
-      </c>
-      <c r="E10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Настройка СУБД сводится к нескольким параметрам: расположение файлов, память, журнал и сетевой доступ. Разбирается, что менять и как проверить результат.</t>
-        </is>
-      </c>
-      <c r="F10" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">конфигурация, параметр, кэш, журнал, порт, перезапуск</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">6</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C11" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 4. Пользователи и роли</t>
-        </is>
-      </c>
-      <c r="D11" s="6">
-        <v>2</v>
-      </c>
-      <c r="E11" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Доступ к данным строится на ролях, а не на отдельных аккаунтах. Разбираются привилегии, владение объектами и проверка выданных прав.</t>
-        </is>
-      </c>
-      <c r="F11" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">привилегия, владелец объекта, схема, GRANT, аудит прав, наследование ролей</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="45" customHeight="1">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">7-8</t>
+          <t xml:space="preserve">7</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 3. Резервное копирование; Восстановление</t>
+          <t xml:space="preserve">Лекция 5. Резервное копирование</t>
         </is>
       </c>
       <c r="D12" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты делают полную и инкрементную копию учебной базы и восстанавливают её на чистом месте. Сдают скрипты копирования и протокол восстановления с проверкой данных.</t>
+          <t xml:space="preserve">Копия нужна не для отчёта, а для восстановления в срок. Разбираются виды копий, расписание, хранение и проверка пригодности копии к восстановлению.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">полная копия, инкремент, точка восстановления, проверка данных, протокол, чистое место</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="45" customHeight="1">
+          <t xml:space="preserve">полная копия, дифференциальная копия, инкремент, расписание, хранение, проверка копии</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="60" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">9</t>
+          <t xml:space="preserve">8</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -397,7 +397,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 5. Резервное копирование</t>
+          <t xml:space="preserve">Лекция 6. Восстановление</t>
         </is>
       </c>
       <c r="D13" s="6">
@@ -405,119 +405,119 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Копия нужна не для отчёта, а для восстановления в срок. Разбираются виды копий, расписание, хранение и проверка пригодности копии к восстановлению.</t>
+          <t xml:space="preserve">Восстановление возвращает базу к нужному моменту, а не просто к последней копии. Разбираются полное и точечное восстановление и порядок применения журналов.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">полная копия, дифференциальная копия, инкремент, расписание, хранение, проверка копии</t>
+          <t xml:space="preserve">журнал, целостность, точка отказа, порядок применения, проверка данных</t>
         </is>
       </c>
     </row>
     <row r="14" ht="60" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">10</t>
+          <t xml:space="preserve">9-10</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 6. Восстановление</t>
+          <t xml:space="preserve">Практика 3. Резервное копирование; Восстановление</t>
         </is>
       </c>
       <c r="D14" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Восстановление возвращает базу к нужному моменту, а не просто к последней копии. Разбираются полное и точечное восстановление и порядок применения журналов.</t>
+          <t xml:space="preserve">Студенты делают полную и инкрементную копию учебной базы и восстанавливают её на чистом месте. Сдают скрипты копирования и протокол восстановления с проверкой данных.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">журнал, целостность, точка отказа, порядок применения, проверка данных</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="60" customHeight="1">
+          <t xml:space="preserve">полная копия, инкремент, точка восстановления, проверка данных, протокол, чистое место</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="45" customHeight="1">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">11-12</t>
+          <t xml:space="preserve">11</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 4. Индексы; Оптимизация запроса</t>
+          <t xml:space="preserve">Лекция 7. Репликация</t>
         </is>
       </c>
       <c r="D15" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты добавляют индексы к учебной базе и сравнивают планы запросов до и после. Сдают SQL-скрипты индексов и замеры времени выполнения.</t>
+          <t xml:space="preserve">Репликация держит копии базы на нескольких узлах и распределяет чтение. Разбираются ведущий и ведомый узлы, отставание и конфликты записи.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">план запроса, полное сканирование, селективность, время выполнения, замер, составной ключ</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="45" customHeight="1">
+          <t xml:space="preserve">ведущий узел, ведомый узел, отставание, конфликт записи, журнал изменений, переключение</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="60" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
+          <t xml:space="preserve">12</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 8. Индексы и производительность</t>
+        </is>
+      </c>
+      <c r="D16" s="6">
+        <v>2</v>
+      </c>
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Индекс ускоряет чтение и замедляет запись, поэтому его строят под конкретный запрос. Разбираются виды индексов, селективность и цена поддержки.</t>
+        </is>
+      </c>
+      <c r="F16" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">B-дерево, порядок столбцов, селективность, покрытие запроса, стоимость записи, статистика</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
           <t xml:space="preserve">13</t>
         </is>
       </c>
-      <c r="B16" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 7. Репликация</t>
-        </is>
-      </c>
-      <c r="D16" s="6">
-        <v>2</v>
-      </c>
-      <c r="E16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Репликация держит копии базы на нескольких узлах и распределяет чтение. Разбираются ведущий и ведомый узлы, отставание и конфликты записи.</t>
-        </is>
-      </c>
-      <c r="F16" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">ведущий узел, ведомый узел, отставание, конфликт записи, журнал изменений, переключение</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="60" customHeight="1">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">14</t>
-        </is>
-      </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 5. Транзакции</t>
+          <t xml:space="preserve">Лекция 9. Оптимизация запросов</t>
         </is>
       </c>
       <c r="D17" s="6">
@@ -525,46 +525,46 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты проверяют свойства транзакций на учебной базе: фиксацию, откат и изоляцию параллельных изменений. Сдают SQL-скрипты сценариев и таблицу наблюдений.</t>
+          <t xml:space="preserve">Медленный запрос обычно вызван лишним сканированием, плохим соединением или недостатком статистики. Разбирается чтение плана и порядок исправления.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">фиксация, откат, уровень изоляции, параллельная сессия, ACID, блокировка</t>
+          <t xml:space="preserve">план выполнения, соединение, сканирование, статистика, подзапрос, время отклика</t>
         </is>
       </c>
     </row>
     <row r="18" ht="60" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">15</t>
+          <t xml:space="preserve">14-15</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 8. Индексы и производительность</t>
+          <t xml:space="preserve">Практика 4. Индексы; Оптимизация запроса</t>
         </is>
       </c>
       <c r="D18" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Индекс ускоряет чтение и замедляет запись, поэтому его строят под конкретный запрос. Разбираются виды индексов, селективность и цена поддержки.</t>
+          <t xml:space="preserve">Студенты добавляют индексы к учебной базе и сравнивают планы запросов до и после. Сдают SQL-скрипты индексов и замеры времени выполнения.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-дерево, порядок столбцов, селективность, покрытие запроса, стоимость записи, статистика</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="45" customHeight="1">
+          <t xml:space="preserve">план запроса, полное сканирование, селективность, время выполнения, замер, составной ключ</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">16</t>
@@ -572,12 +572,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 6. Импорт JSON</t>
+          <t xml:space="preserve">Лекция 10. Транзакции и блокировки</t>
         </is>
       </c>
       <c r="D19" s="6">
@@ -585,16 +585,16 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты загружают данные из JSON в таблицы учебной базы и проверяют результат запросами. Сдают скрипт импорта и отчёт о числе загруженных строк.</t>
+          <t xml:space="preserve">Транзакции удерживают данные согласованными, а блокировки решают, кто и когда меняет строку. Разбираются уровни изоляции, взаимные блокировки и откат.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">разбор структуры, тип данных, проверка строк, скрипт, кодировка, связь таблиц</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="45" customHeight="1">
+          <t xml:space="preserve">уровень изоляции, взаимная блокировка, ожидание, откат, долгая транзакция, фиксация</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="60" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">17</t>
@@ -602,12 +602,12 @@
       </c>
       <c r="B20" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 9. Оптимизация запросов</t>
+          <t xml:space="preserve">Практика 5. Транзакции</t>
         </is>
       </c>
       <c r="D20" s="6">
@@ -615,12 +615,12 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Медленный запрос обычно вызван лишним сканированием, плохим соединением или недостатком статистики. Разбирается чтение плана и порядок исправления.</t>
+          <t xml:space="preserve">Студенты проверяют свойства транзакций на учебной базе: фиксацию, откат и изоляцию параллельных изменений. Сдают SQL-скрипты сценариев и таблицу наблюдений.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">план выполнения, соединение, сканирование, статистика, подзапрос, время отклика</t>
+          <t xml:space="preserve">фиксация, откат, уровень изоляции, параллельная сессия, ACID, блокировка</t>
         </is>
       </c>
     </row>
@@ -632,12 +632,12 @@
       </c>
       <c r="B21" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 7. Экспорт</t>
+          <t xml:space="preserve">Лекция 11. Импорт и экспорт</t>
         </is>
       </c>
       <c r="D21" s="6">
@@ -645,16 +645,16 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты выгружают данные учебной базы в файл для обмена и проверяют выгрузку обратной загрузкой. Сдают скрипт экспорта и отчёт о сверке строк.</t>
+          <t xml:space="preserve">Обмен данными требует договорённости о формате, кодировке и правилах ошибок. Разбираются CSV и JSON, пакетная загрузка и проверка целостности.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">формат обмена, CSV, кодировка, сверка, выборка, файл</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="60" customHeight="1">
+          <t xml:space="preserve">CSV, JSON, кодировка, пакетная загрузка, ошибка строки, целостность</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="45" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">19</t>
@@ -662,12 +662,12 @@
       </c>
       <c r="B22" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 10. Транзакции и блокировки</t>
+          <t xml:space="preserve">Практика 6. Импорт JSON</t>
         </is>
       </c>
       <c r="D22" s="6">
@@ -675,12 +675,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Транзакции удерживают данные согласованными, а блокировки решают, кто и когда меняет строку. Разбираются уровни изоляции, взаимные блокировки и откат.</t>
+          <t xml:space="preserve">Студенты загружают данные из JSON в таблицы учебной базы и проверяют результат запросами. Сдают скрипт импорта и отчёт о числе загруженных строк.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">уровень изоляции, взаимная блокировка, ожидание, откат, долгая транзакция, фиксация</t>
+          <t xml:space="preserve">разбор структуры, тип данных, проверка строк, скрипт, кодировка, связь таблиц</t>
         </is>
       </c>
     </row>
@@ -697,117 +697,117 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">Практика 7. Экспорт</t>
+        </is>
+      </c>
+      <c r="D23" s="6">
+        <v>2</v>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Студенты выгружают данные учебной базы в файл для обмена и проверяют выгрузку обратной загрузкой. Сдают скрипт экспорта и отчёт о сверке строк.</t>
+        </is>
+      </c>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">формат обмена, CSV, кодировка, сверка, выборка, файл</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="60" customHeight="1">
+      <c r="A24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">21</t>
+        </is>
+      </c>
+      <c r="B24" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Лекция 12. Автоматизация скриптов</t>
+        </is>
+      </c>
+      <c r="D24" s="6">
+        <v>2</v>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Автоматизация убирает ручные шаги из обслуживания базы и делает их повторяемыми. Разбираются параметры скрипта, журналирование и безопасный повторный запуск.</t>
+        </is>
+      </c>
+      <c r="F24" s="5" t="inlineStr">
+        <is>
+          <t xml:space="preserve">параметр, журнал, код возврата, повторный запуск, обработка ошибок, расписание</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="45" customHeight="1">
+      <c r="A25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">22</t>
+        </is>
+      </c>
+      <c r="B25" s="6" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Практика</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
           <t xml:space="preserve">Практика 8. Скрипт автоматизации</t>
         </is>
       </c>
-      <c r="D23" s="6">
-        <v>2</v>
-      </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="D25" s="6">
+        <v>2</v>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">Студенты пишут скрипт, который создаёт таблицы, загружает данные и делает копию без ручных шагов. Сдают скрипт с проверкой запуска на чистой базе.</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F25" s="5" t="inlineStr">
         <is>
           <t xml:space="preserve">идемпотентность, схема, загрузка данных, повторный запуск, проверка, командный файл</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="45" customHeight="1">
-      <c r="A24" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">21</t>
-        </is>
-      </c>
-      <c r="B24" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 11. Импорт и экспорт</t>
-        </is>
-      </c>
-      <c r="D24" s="6">
-        <v>2</v>
-      </c>
-      <c r="E24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Обмен данными требует договорённости о формате, кодировке и правилах ошибок. Разбираются CSV и JSON, пакетная загрузка и проверка целостности.</t>
-        </is>
-      </c>
-      <c r="F24" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">CSV, JSON, кодировка, пакетная загрузка, ошибка строки, целостность</t>
-        </is>
-      </c>
-    </row>
-    <row r="25" ht="60" customHeight="1">
-      <c r="A25" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">22</t>
-        </is>
-      </c>
-      <c r="B25" s="6" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция</t>
-        </is>
-      </c>
-      <c r="C25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Лекция 12. Автоматизация скриптов</t>
-        </is>
-      </c>
-      <c r="D25" s="6">
-        <v>2</v>
-      </c>
-      <c r="E25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Автоматизация убирает ручные шаги из обслуживания базы и делает их повторяемыми. Разбираются параметры скрипта, журналирование и безопасный повторный запуск.</t>
-        </is>
-      </c>
-      <c r="F25" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">параметр, журнал, код возврата, повторный запуск, обработка ошибок, расписание</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="60" customHeight="1">
+    <row r="26" ht="45" customHeight="1">
       <c r="A26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">23-24</t>
+          <t xml:space="preserve">23</t>
         </is>
       </c>
       <c r="B26" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 9. Планировщик; Мониторинг</t>
+          <t xml:space="preserve">Лекция 13. Планировщик заданий</t>
         </is>
       </c>
       <c r="D26" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты ставят скрипт обслуживания в планировщик и настраивают сбор метрик учебной базы. Сдают задание планировщика, скрипт метрик и отчёт наблюдений.</t>
+          <t xml:space="preserve">Планировщик запускает обслуживание базы без участия человека. Разбираются расписание, права запуска, журнал и обработка сбоя задания.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">расписание, метрика, журнал запуска, соединение, наблюдение, порог</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="45" customHeight="1">
+          <t xml:space="preserve">расписание, задание, права запуска, журнал, сбой, учётная запись службы</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="60" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">25</t>
+          <t xml:space="preserve">24</t>
         </is>
       </c>
       <c r="B27" s="6" t="inlineStr">
@@ -817,7 +817,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 13. Планировщик заданий</t>
+          <t xml:space="preserve">Лекция 14. Мониторинг</t>
         </is>
       </c>
       <c r="D27" s="6">
@@ -825,79 +825,79 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Планировщик запускает обслуживание базы без участия человека. Разбираются расписание, права запуска, журнал и обработка сбоя задания.</t>
+          <t xml:space="preserve">Мониторинг отвечает, что с базой сейчас и что изменится через неделю. Разбираются метрики, пороги оповещений и разбор инцидента по данным наблюдения.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">расписание, задание, права запуска, журнал, сбой, учётная запись службы</t>
+          <t xml:space="preserve">метрика, порог, оповещение, журнал, нагрузка, инцидент</t>
         </is>
       </c>
     </row>
     <row r="28" ht="60" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">26</t>
+          <t xml:space="preserve">25-26</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 14. Мониторинг</t>
+          <t xml:space="preserve">Практика 9. Планировщик; Мониторинг</t>
         </is>
       </c>
       <c r="D28" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мониторинг отвечает, что с базой сейчас и что изменится через неделю. Разбираются метрики, пороги оповещений и разбор инцидента по данным наблюдения.</t>
+          <t xml:space="preserve">Студенты ставят скрипт обслуживания в планировщик и настраивают сбор метрик учебной базы. Сдают задание планировщика, скрипт метрик и отчёт наблюдений.</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">метрика, порог, оповещение, журнал, нагрузка, инцидент</t>
-        </is>
-      </c>
-    </row>
-    <row r="29" ht="60" customHeight="1">
+          <t xml:space="preserve">расписание, метрика, журнал запуска, соединение, наблюдение, порог</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="45" customHeight="1">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">27-28</t>
+          <t xml:space="preserve">27</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика</t>
+          <t xml:space="preserve">Лекция</t>
         </is>
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 10. Аудит; Безопасность</t>
+          <t xml:space="preserve">Лекция 15. Аудит</t>
         </is>
       </c>
       <c r="D29" s="6">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты включают аудит действий в учебной базе и проверяют защиту доступа, секретов и копий. Сдают настройки аудита, выгрузку событий и список рисков.</t>
+          <t xml:space="preserve">Аудит фиксирует, кто и что сделал с данными, и помогает разобрать инцидент. Разбираются события, хранение журнала и разграничение доступа к нему.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">событие, журнал доступа, секрет, права, риск, мера защиты</t>
+          <t xml:space="preserve">событие, журнал, политика, хранение, разбор инцидента, подотчётность</t>
         </is>
       </c>
     </row>
     <row r="30" ht="45" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">29</t>
+          <t xml:space="preserve">28</t>
         </is>
       </c>
       <c r="B30" s="6" t="inlineStr">
@@ -907,7 +907,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 15. Аудит</t>
+          <t xml:space="preserve">Лекция 16. Безопасность</t>
         </is>
       </c>
       <c r="D30" s="6">
@@ -915,19 +915,19 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аудит фиксирует, кто и что сделал с данными, и помогает разобрать инцидент. Разбираются события, хранение журнала и разграничение доступа к нему.</t>
+          <t xml:space="preserve">Безопасность базы строится на минимальных правах, защите секретов и контроле доступа к копиям. Разбираются типовые атаки и меры защиты данных.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">событие, журнал, политика, хранение, разбор инцидента, подотчётность</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="45" customHeight="1">
+          <t xml:space="preserve">привилегия, строка подключения, секрет, шифрование, инъекция, доступ к копиям</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="60" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">30</t>
+          <t xml:space="preserve">29-30</t>
         </is>
       </c>
       <c r="B31" s="6" t="inlineStr">
@@ -937,20 +937,20 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 11. Миграция</t>
+          <t xml:space="preserve">Практика 10. Аудит; Безопасность</t>
         </is>
       </c>
       <c r="D31" s="6">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты переносят учебную базу на новую версию схемы с сохранением данных. Сдают скрипты миграции и отката и отчёт о проверке данных.</t>
+          <t xml:space="preserve">Студенты включают аудит действий в учебной базе и проверяют защиту доступа, секретов и копий. Сдают настройки аудита, выгрузку событий и список рисков.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">версия схемы, откат, перенос данных, проверка, скрипт, совместимость</t>
+          <t xml:space="preserve">событие, журнал доступа, секрет, права, риск, мера защиты</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 16. Безопасность</t>
+          <t xml:space="preserve">Лекция 17. Миграции</t>
         </is>
       </c>
       <c r="D32" s="6">
@@ -975,12 +975,12 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Безопасность базы строится на минимальных правах, защите секретов и контроле доступа к копиям. Разбираются типовые атаки и меры защиты данных.</t>
+          <t xml:space="preserve">Миграция меняет схему на работающей базе без остановки и потери данных. Разбираются версии, прямой и обратный скрипт, проверка и порядок выпуска.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">привилегия, строка подключения, секрет, шифрование, инъекция, доступ к копиям</t>
+          <t xml:space="preserve">версия, обратный скрипт, совместимость, проверка, выпуск, окно обслуживания</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 12. Итоговая БД</t>
+          <t xml:space="preserve">Практика 11. Миграция</t>
         </is>
       </c>
       <c r="D33" s="6">
@@ -1005,12 +1005,12 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты собирают учебную базу целиком: схема, роли, индексы, копия и скрипт обслуживания. Сдают базу и комплект скриптов с протоколом проверки.</t>
+          <t xml:space="preserve">Студенты переносят учебную базу на новую версию схемы с сохранением данных. Сдают скрипты миграции и отката и отчёт о проверке данных.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">схема, ограничение, роль, индекс, копия, чек-лист</t>
+          <t xml:space="preserve">версия схемы, откат, перенос данных, проверка, скрипт, совместимость</t>
         </is>
       </c>
     </row>
@@ -1022,12 +1022,12 @@
       </c>
       <c r="B34" s="6" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция</t>
+          <t xml:space="preserve">Практика</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 17. Миграции</t>
+          <t xml:space="preserve">Практика 12. Итоговая БД</t>
         </is>
       </c>
       <c r="D34" s="6">
@@ -1035,12 +1035,12 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Миграция меняет схему на работающей базе без остановки и потери данных. Разбираются версии, прямой и обратный скрипт, проверка и порядок выпуска.</t>
+          <t xml:space="preserve">Студенты собирают учебную базу целиком: схема, роли, индексы, копия и скрипт обслуживания. Сдают базу и комплект скриптов с протоколом проверки.</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">версия, обратный скрипт, совместимость, проверка, выпуск, окно обслуживания</t>
+          <t xml:space="preserve">схема, ограничение, роль, индекс, копия, чек-лист</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rework database automation around MySQL, XAMPP and .NET 10
MДК.07.01 no longer uses PostgreSQL in a virtual machine. The plan and all 29 lessons now use MySQL from XAMPP, phpMyAdmin with utf8mb4, .NET SDK 10, MySqlConnector and Visual Studio 2022 with the .NET desktop workload. Discipline cards drop the СПО label and hours, keeping the lesson count and exam or credit.
</commit_message>
<xml_diff>
--- a/courses/4/db-automation/dist/Учебный_план_Управление_и_автоматизация_баз_данных.xlsx
+++ b/courses/4/db-automation/dist/Учебный_план_Управление_и_автоматизация_баз_данных.xlsx
@@ -187,7 +187,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 1. Управление и автоматизация БД</t>
+          <t xml:space="preserve">Управление и автоматизация БД</t>
         </is>
       </c>
       <c r="D6" s="6">
@@ -195,16 +195,16 @@
       </c>
       <c r="E6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Администратор БД отвечает за доступ, сохранность и скорость работы данных. Разбираются зоны ответственности, регламентные задачи и границы автоматизации.</t>
+          <t xml:space="preserve">Администратор MySQL отвечает за доступ, сохранность и скорость данных, а автоматизация на C# убирает ручные шаги. Разбираются роли, регламент и инструменты XAMPP, Visual Studio и .NET SDK 10.</t>
         </is>
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">администратор БД, регламент, обслуживание, доступность, зона ответственности</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="60" customHeight="1">
+          <t xml:space="preserve">администратор БД, XAMPP, MySQL, регламент, автоматизация, .NET SDK 10</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="45" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">2</t>
@@ -217,7 +217,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 2. Архитектура PostgreSQL</t>
+          <t xml:space="preserve">Архитектура MySQL и InnoDB</t>
         </is>
       </c>
       <c r="D7" s="6">
@@ -225,12 +225,12 @@
       </c>
       <c r="E7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PostgreSQL делится на процессы, разделяемую память и файлы WAL; от этой раскладки зависит поведение запросов. Разбираются клиент-серверная и файловая модели.</t>
+          <t xml:space="preserve">MySQL в XAMPP состоит из сервера, InnoDB, буферного пула и журналов. Разбирается, как устроены таблицы, транзакции и восстановление после сбоя.</t>
         </is>
       </c>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ядро, клиент-сервер, буферный кэш, журнал, файл данных, процесс</t>
+          <t xml:space="preserve">MySQL, InnoDB, буферный пул, redo log, undo log, binary log</t>
         </is>
       </c>
     </row>
@@ -247,7 +247,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 3. Установка и настройка PostgreSQL</t>
+          <t xml:space="preserve">XAMPP, MySQL и подключение из .NET</t>
         </is>
       </c>
       <c r="D8" s="6">
@@ -255,16 +255,16 @@
       </c>
       <c r="E8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Настройка PostgreSQL сводится к расположению файлов, памяти, WAL и сетевому доступу. Разбирается, что менять и как проверить результат после перезапуска.</t>
+          <t xml:space="preserve">XAMPP запускает Apache и MySQL, phpMyAdmin даёт браузерный доступ, а .NET подключается к базе через MySqlConnector. Разбирается установка, кодировка utf8mb4 и строка подключения.</t>
         </is>
       </c>
       <c r="F8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">конфигурация, параметр, кэш, журнал, порт, перезапуск</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="60" customHeight="1">
+          <t xml:space="preserve">XAMPP, phpMyAdmin, utf8mb4, MySqlConnector, строка подключения, порт 3306</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="45" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">4</t>
@@ -277,7 +277,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 1. Установка PostgreSQL и подключение</t>
+          <t xml:space="preserve">Запуск XAMPP, база utf8mb4, подключение из .NET</t>
         </is>
       </c>
       <c r="D9" s="6">
@@ -285,12 +285,12 @@
       </c>
       <c r="E9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты устанавливают PostgreSQL в учебной Linux VM, создают учебную базу и подключаются к ней через psql. Сдают протокол установки, список баз и проверку подключения.</t>
+          <t xml:space="preserve">Запускают MySQL в XAMPP, создают базу dean в phpMyAdmin с utf8mb4, подключаются из консольного приложения .NET SDK 10 и сдают протокол.</t>
         </is>
       </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">PostgreSQL, VirtualBox, psql, createdb, подключение, порт 5432</t>
+          <t xml:space="preserve">XAMPP, phpMyAdmin, utf8mb4, MySqlConnector, .NET SDK 10, порт 3306</t>
         </is>
       </c>
     </row>
@@ -307,7 +307,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 4. Пользователи и роли</t>
+          <t xml:space="preserve">Пользователи и роли MySQL</t>
         </is>
       </c>
       <c r="D10" s="6">
@@ -315,16 +315,16 @@
       </c>
       <c r="E10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Доступ к данным строится на ролях, а не на отдельных аккаунтах. Разбираются привилегии, владение объектами и проверка выданных прав.</t>
+          <t xml:space="preserve">Доступ к MySQL строится на пользователях, ролях и привилегиях. Разбираются GRANT, REVOKE, роли MySQL 8 и проверка прав из приложения.</t>
         </is>
       </c>
       <c r="F10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">привилегия, владелец объекта, схема, GRANT, аудит прав, наследование ролей</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="60" customHeight="1">
+          <t xml:space="preserve">пользователь, роль, GRANT, REVOKE, привилегия, минимальные права</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="45" customHeight="1">
       <c r="A11" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">6</t>
@@ -337,7 +337,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 2. Пользователи и роли</t>
+          <t xml:space="preserve">Роли и доступ в MySQL</t>
         </is>
       </c>
       <c r="D11" s="6">
@@ -345,12 +345,12 @@
       </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты создают пользователей учебной базы, выдают права через роли и проверяют доступ от каждого аккаунта. Сдают SQL-скрипт с ролями и таблицу проверки прав.</t>
+          <t xml:space="preserve">Создают пользователей и роли MySQL, выдают минимальные права и проверяют доступ из phpMyAdmin и .NET. Сдают SQL-скрипт и матрицу прав.</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">привилегия, GRANT, REVOKE, минимальные привилегии, учётная запись, проверка доступа</t>
+          <t xml:space="preserve">роль, пользователь, GRANT, REVOKE, матрица прав, проверка</t>
         </is>
       </c>
     </row>
@@ -367,7 +367,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 5. Резервное копирование</t>
+          <t xml:space="preserve">Резервное копирование MySQL</t>
         </is>
       </c>
       <c r="D12" s="6">
@@ -375,12 +375,12 @@
       </c>
       <c r="E12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Копия нужна не для отчёта, а для восстановления в срок. Разбираются виды копий, расписание, хранение и проверка пригодности копии к восстановлению.</t>
+          <t xml:space="preserve">Копия MySQL нужна для восстановления в срок. Разбираются mysqldump, phpMyAdmin Export, binary logs, расписание и проверка копии.</t>
         </is>
       </c>
       <c r="F12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">полная копия, дифференциальная копия, инкремент, расписание, хранение, проверка копии</t>
+          <t xml:space="preserve">mysqldump, phpMyAdmin, binary log, RPO, RTO, проверка копии</t>
         </is>
       </c>
     </row>
@@ -397,7 +397,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 6. Восстановление</t>
+          <t xml:space="preserve">Восстановление и журналы MySQL</t>
         </is>
       </c>
       <c r="D13" s="6">
@@ -405,16 +405,16 @@
       </c>
       <c r="E13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Восстановление возвращает базу к нужному моменту, а не просто к последней копии. Разбираются полное и точечное восстановление и порядок применения журналов.</t>
+          <t xml:space="preserve">Восстановление MySQL возвращает базу к нужному моменту с помощью дампа и binary log. Разбираются импорт, mysqlbinlog, проверка целостности и порядок действий.</t>
         </is>
       </c>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">журнал, целостность, точка отказа, порядок применения, проверка данных</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="60" customHeight="1">
+          <t xml:space="preserve">mysql, mysqlbinlog, point-in-time, импорт, целостность, проверка</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="45" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">9-10</t>
@@ -427,7 +427,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 3. Резервное копирование; Восстановление</t>
+          <t xml:space="preserve">Резервное копирование и восстановление</t>
         </is>
       </c>
       <c r="D14" s="6">
@@ -435,12 +435,12 @@
       </c>
       <c r="E14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты делают полную и инкрементную копию учебной базы и восстанавливают её на чистом месте. Сдают скрипты копирования и протокол восстановления с проверкой данных.</t>
+          <t xml:space="preserve">Делают дамп mysqldump и экспорт phpMyAdmin, восстанавливают базу и проверяют binary log. Сдают скрипты и протокол сверки.</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">полная копия, инкремент, точка восстановления, проверка данных, протокол, чистое место</t>
+          <t xml:space="preserve">mysqldump, phpMyAdmin, восстановление, binary log, сверка, протокол</t>
         </is>
       </c>
     </row>
@@ -457,7 +457,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 7. Репликация</t>
+          <t xml:space="preserve">Репликация MySQL</t>
         </is>
       </c>
       <c r="D15" s="6">
@@ -465,12 +465,12 @@
       </c>
       <c r="E15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Репликация держит копии базы на нескольких узлах и распределяет чтение. Разбираются ведущий и ведомый узлы, отставание и конфликты записи.</t>
+          <t xml:space="preserve">Репликация MySQL держит копию на втором узле и распределяет чтение. Разбираются source/replica, binary log, отставание и переключение.</t>
         </is>
       </c>
       <c r="F15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">ведущий узел, ведомый узел, отставание, конфликт записи, журнал изменений, переключение</t>
+          <t xml:space="preserve">репликация, source, replica, binary log, лаг, failover</t>
         </is>
       </c>
     </row>
@@ -487,7 +487,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 8. Индексы и производительность</t>
+          <t xml:space="preserve">Индексы и производительность InnoDB</t>
         </is>
       </c>
       <c r="D16" s="6">
@@ -495,12 +495,12 @@
       </c>
       <c r="E16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Индекс ускоряет чтение и замедляет запись, поэтому его строят под конкретный запрос. Разбираются виды индексов, селективность и цена поддержки.</t>
+          <t xml:space="preserve">Индекс InnoDB ускоряет чтение и замедляет запись. Разбираются B-tree, составной индекс, селективность, покрывающий и частичный индекс.</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">B-дерево, порядок столбцов, селективность, покрытие запроса, стоимость записи, статистика</t>
+          <t xml:space="preserve">B-tree, составной индекс, селективность, покрывающий индекс, SHOW INDEX, стоимость записи</t>
         </is>
       </c>
     </row>
@@ -517,7 +517,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 9. Оптимизация запросов</t>
+          <t xml:space="preserve">Оптимизация запросов MySQL</t>
         </is>
       </c>
       <c r="D17" s="6">
@@ -525,16 +525,16 @@
       </c>
       <c r="E17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Медленный запрос обычно вызван лишним сканированием, плохим соединением или недостатком статистики. Разбирается чтение плана и порядок исправления.</t>
+          <t xml:space="preserve">Медленный запрос MySQL лечится по EXPLAIN и статистике. Разбираются типы соединений, сканирования, сортировки и порядок оптимизации.</t>
         </is>
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">план выполнения, соединение, сканирование, статистика, подзапрос, время отклика</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="60" customHeight="1">
+          <t xml:space="preserve">EXPLAIN, JOIN, сканирование, статистика, ANALYZE TABLE, время отклика</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="45" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">14-15</t>
@@ -547,7 +547,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 4. Индексы; Оптимизация запроса</t>
+          <t xml:space="preserve">Индексы и оптимизация</t>
         </is>
       </c>
       <c r="D18" s="6">
@@ -555,16 +555,16 @@
       </c>
       <c r="E18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты добавляют индексы к учебной базе и сравнивают планы запросов до и после. Сдают SQL-скрипты индексов и замеры времени выполнения.</t>
+          <t xml:space="preserve">Создают большую таблицу, сравнивают EXPLAIN до и после индексов, добавляют составной и покрывающий индекс. Сдают планы и замеры.</t>
         </is>
       </c>
       <c r="F18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">план запроса, полное сканирование, селективность, время выполнения, замер, составной ключ</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="60" customHeight="1">
+          <t xml:space="preserve">EXPLAIN, индекс, селективность, покрывающий индекс, ANALYZE TABLE, замер</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="45" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">16</t>
@@ -577,7 +577,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 10. Транзакции и блокировки</t>
+          <t xml:space="preserve">Транзакции и блокировки InnoDB</t>
         </is>
       </c>
       <c r="D19" s="6">
@@ -585,16 +585,16 @@
       </c>
       <c r="E19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Транзакции удерживают данные согласованными, а блокировки решают, кто и когда меняет строку. Разбираются уровни изоляции, взаимные блокировки и откат.</t>
+          <t xml:space="preserve">Транзакции InnoDB удерживают согласованность, а блокировки решают, кто меняет строку. Разбираются уровни изоляции, deadlock и долгие транзакции.</t>
         </is>
       </c>
       <c r="F19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">уровень изоляции, взаимная блокировка, ожидание, откат, долгая транзакция, фиксация</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="60" customHeight="1">
+          <t xml:space="preserve">InnoDB, транзакция, изоляция, deadlock, блокировка, performance_schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="45" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">17</t>
@@ -607,7 +607,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 5. Транзакции</t>
+          <t xml:space="preserve">Транзакции</t>
         </is>
       </c>
       <c r="D20" s="6">
@@ -615,12 +615,12 @@
       </c>
       <c r="E20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты проверяют свойства транзакций на учебной базе: фиксацию, откат и изоляцию параллельных изменений. Сдают SQL-скрипты сценариев и таблицу наблюдений.</t>
+          <t xml:space="preserve">Проверяют транзакции и блокировки InnoDB в двух сессиях, вызывают deadlock и читают performance_schema. Сдают наблюдения.</t>
         </is>
       </c>
       <c r="F20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">фиксация, откат, уровень изоляции, параллельная сессия, ACID, блокировка</t>
+          <t xml:space="preserve">START TRANSACTION, COMMIT, ROLLBACK, изоляция, deadlock, performance_schema</t>
         </is>
       </c>
     </row>
@@ -637,7 +637,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 11. Импорт и экспорт</t>
+          <t xml:space="preserve">Импорт и экспорт данных</t>
         </is>
       </c>
       <c r="D21" s="6">
@@ -645,12 +645,12 @@
       </c>
       <c r="E21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Обмен данными требует договорённости о формате, кодировке и правилах ошибок. Разбираются CSV и JSON, пакетная загрузка и проверка целостности.</t>
+          <t xml:space="preserve">Обмен данными MySQL требует формата, кодировки и правил ошибок. Разбираются CSV, JSON, LOAD DATA, phpMyAdmin Import и проверка строк.</t>
         </is>
       </c>
       <c r="F21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">CSV, JSON, кодировка, пакетная загрузка, ошибка строки, целостность</t>
+          <t xml:space="preserve">CSV, JSON, LOAD DATA, phpMyAdmin, utf8mb4, сверка строк</t>
         </is>
       </c>
     </row>
@@ -667,7 +667,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 6. Импорт JSON</t>
+          <t xml:space="preserve">Импорт JSON</t>
         </is>
       </c>
       <c r="D22" s="6">
@@ -675,12 +675,12 @@
       </c>
       <c r="E22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты загружают данные из JSON в таблицы учебной базы и проверяют результат запросами. Сдают скрипт импорта и отчёт о числе загруженных строк.</t>
+          <t xml:space="preserve">Загружают JSON в MySQL через phpMyAdmin и .NET, проверяют utf8mb4, типы и связи. Сдают скрипт и отчёт о строках.</t>
         </is>
       </c>
       <c r="F22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">разбор структуры, тип данных, проверка строк, скрипт, кодировка, связь таблиц</t>
+          <t xml:space="preserve">JSON, phpMyAdmin, utf8mb4, MySqlConnector, проверка, связи</t>
         </is>
       </c>
     </row>
@@ -697,7 +697,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 7. Экспорт</t>
+          <t xml:space="preserve">Экспорт</t>
         </is>
       </c>
       <c r="D23" s="6">
@@ -705,12 +705,12 @@
       </c>
       <c r="E23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты выгружают данные учебной базы в файл для обмена и проверяют выгрузку обратной загрузкой. Сдают скрипт экспорта и отчёт о сверке строк.</t>
+          <t xml:space="preserve">Выгружают данные MySQL в CSV и JSON, проверяют кодировку и обратную загрузку. Сдают скрипты и сверку.</t>
         </is>
       </c>
       <c r="F23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">формат обмена, CSV, кодировка, сверка, выборка, файл</t>
+          <t xml:space="preserve">CSV, JSON, экспорт, utf8mb4, сверка, файл</t>
         </is>
       </c>
     </row>
@@ -727,7 +727,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 12. Автоматизация скриптов</t>
+          <t xml:space="preserve">Автоматизация на C# и .NET SDK 10</t>
         </is>
       </c>
       <c r="D24" s="6">
@@ -735,12 +735,12 @@
       </c>
       <c r="E24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Автоматизация убирает ручные шаги из обслуживания базы и делает их повторяемыми. Разбираются параметры скрипта, журналирование и безопасный повторный запуск.</t>
+          <t xml:space="preserve">Автоматизация на C# и .NET SDK 10 делает обслуживание MySQL повторяемым. Разбираются консольное приложение, MySqlConnector, аргументы, журнал и коды возврата.</t>
         </is>
       </c>
       <c r="F24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">параметр, журнал, код возврата, повторный запуск, обработка ошибок, расписание</t>
+          <t xml:space="preserve">.NET SDK 10, C#, MySqlConnector, консольное приложение, журнал, код возврата</t>
         </is>
       </c>
     </row>
@@ -757,7 +757,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 8. Скрипт автоматизации</t>
+          <t xml:space="preserve">Консольное приложение обслуживания</t>
         </is>
       </c>
       <c r="D25" s="6">
@@ -765,12 +765,12 @@
       </c>
       <c r="E25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты пишут скрипт, который создаёт таблицы, загружает данные и делает копию без ручных шагов. Сдают скрипт с проверкой запуска на чистой базе.</t>
+          <t xml:space="preserve">Пишут консольное приложение .NET SDK 10 для обслуживания MySQL: дамп, проверка, журнал и коды возврата. Запускают дважды.</t>
         </is>
       </c>
       <c r="F25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">идемпотентность, схема, загрузка данных, повторный запуск, проверка, командный файл</t>
+          <t xml:space="preserve">.NET SDK 10, C#, MySqlConnector, дамп, журнал, идемпотентность</t>
         </is>
       </c>
     </row>
@@ -787,7 +787,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 13. Планировщик заданий</t>
+          <t xml:space="preserve">Планировщик заданий и события MySQL</t>
         </is>
       </c>
       <c r="D26" s="6">
@@ -795,16 +795,16 @@
       </c>
       <c r="E26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Планировщик запускает обслуживание базы без участия человека. Разбираются расписание, права запуска, журнал и обработка сбоя задания.</t>
+          <t xml:space="preserve">Планировщик Windows и события MySQL запускают обслуживание без человека. Разбираются Task Scheduler, MySQL Event Scheduler, права и журнал.</t>
         </is>
       </c>
       <c r="F26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">расписание, задание, права запуска, журнал, сбой, учётная запись службы</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="60" customHeight="1">
+          <t xml:space="preserve">Планировщик Windows, Task Scheduler, MySQL Event, расписание, журнал, права</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="45" customHeight="1">
       <c r="A27" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">24</t>
@@ -817,7 +817,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 14. Мониторинг</t>
+          <t xml:space="preserve">Мониторинг MySQL и приложение WinForms</t>
         </is>
       </c>
       <c r="D27" s="6">
@@ -825,16 +825,16 @@
       </c>
       <c r="E27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мониторинг отвечает, что с базой сейчас и что изменится через неделю. Разбираются метрики, пороги оповещений и разбор инцидента по данным наблюдения.</t>
+          <t xml:space="preserve">Мониторинг MySQL отвечает, что с базой сейчас. Разбираются performance_schema, статусы, долгие запросы, блокировки и приложение WinForms.</t>
         </is>
       </c>
       <c r="F27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">метрика, порог, оповещение, журнал, нагрузка, инцидент</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="60" customHeight="1">
+          <t xml:space="preserve">performance_schema, SHOW STATUS, метрика, порог, WinForms, мониторинг</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="45" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">25-26</t>
@@ -847,7 +847,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 9. Планировщик; Мониторинг</t>
+          <t xml:space="preserve">Планировщик и мониторинг</t>
         </is>
       </c>
       <c r="D28" s="6">
@@ -855,12 +855,12 @@
       </c>
       <c r="E28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты ставят скрипт обслуживания в планировщик и настраивают сбор метрик учебной базы. Сдают задание планировщика, скрипт метрик и отчёт наблюдений.</t>
+          <t xml:space="preserve">Ставят приложение обслуживания в Планировщик Windows, собирают метрики MySQL и выводят их в WinForms. Сдают задание, метрики и отчёт.</t>
         </is>
       </c>
       <c r="F28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">расписание, метрика, журнал запуска, соединение, наблюдение, порог</t>
+          <t xml:space="preserve">Task Scheduler, performance_schema, метрика, WinForms, журнал, порог</t>
         </is>
       </c>
     </row>
@@ -877,7 +877,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 15. Аудит</t>
+          <t xml:space="preserve">Аудит MySQL</t>
         </is>
       </c>
       <c r="D29" s="6">
@@ -885,16 +885,16 @@
       </c>
       <c r="E29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аудит фиксирует, кто и что сделал с данными, и помогает разобрать инцидент. Разбираются события, хранение журнала и разграничение доступа к нему.</t>
+          <t xml:space="preserve">Аудит MySQL фиксирует, кто и что сделал. Разбираются general log, триггерная таблица, хранение и защита журнала.</t>
         </is>
       </c>
       <c r="F29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">событие, журнал, политика, хранение, разбор инцидента, подотчётность</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="45" customHeight="1">
+          <t xml:space="preserve">general log, аудит, триггер, журнал, хранение, подотчётность</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="60" customHeight="1">
       <c r="A30" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">28</t>
@@ -907,7 +907,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 16. Безопасность</t>
+          <t xml:space="preserve">Безопасность MySQL и .NET</t>
         </is>
       </c>
       <c r="D30" s="6">
@@ -915,16 +915,16 @@
       </c>
       <c r="E30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Безопасность базы строится на минимальных правах, защите секретов и контроле доступа к копиям. Разбираются типовые атаки и меры защиты данных.</t>
+          <t xml:space="preserve">Безопасность MySQL и .NET строится на минимальных правах, защите строки подключения и проверке ввода. Разбираются SQL-инъекции, секреты и доступ к дампам.</t>
         </is>
       </c>
       <c r="F30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">привилегия, строка подключения, секрет, шифрование, инъекция, доступ к копиям</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="60" customHeight="1">
+          <t xml:space="preserve">привилегия, строка подключения, секрет, SQL-инъекция, параметризованный запрос, дамп</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="45" customHeight="1">
       <c r="A31" s="6" t="inlineStr">
         <is>
           <t xml:space="preserve">29-30</t>
@@ -937,7 +937,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 10. Аудит; Безопасность</t>
+          <t xml:space="preserve">Аудит и безопасность</t>
         </is>
       </c>
       <c r="D31" s="6">
@@ -945,12 +945,12 @@
       </c>
       <c r="E31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты включают аудит действий в учебной базе и проверяют защиту доступа, секретов и копий. Сдают настройки аудита, выгрузку событий и список рисков.</t>
+          <t xml:space="preserve">Включают аудит MySQL, создают триггерную таблицу и проверяют права и секреты. Сдают события, матрицу доступа и риски.</t>
         </is>
       </c>
       <c r="F31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">событие, журнал доступа, секрет, права, риск, мера защиты</t>
+          <t xml:space="preserve">general log, триггер, аудит, привилегия, секрет, риск</t>
         </is>
       </c>
     </row>
@@ -967,7 +967,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Лекция 17. Миграции</t>
+          <t xml:space="preserve">Миграции схемы MySQL</t>
         </is>
       </c>
       <c r="D32" s="6">
@@ -975,12 +975,12 @@
       </c>
       <c r="E32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Миграция меняет схему на работающей базе без остановки и потери данных. Разбираются версии, прямой и обратный скрипт, проверка и порядок выпуска.</t>
+          <t xml:space="preserve">Миграция MySQL меняет схему без потери данных. Разбираются версии, ALTER TABLE, backfill, обратный скрипт и проверка на копии.</t>
         </is>
       </c>
       <c r="F32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">версия, обратный скрипт, совместимость, проверка, выпуск, окно обслуживания</t>
+          <t xml:space="preserve">миграция, schema_version, ALTER TABLE, backfill, rollback, проверка</t>
         </is>
       </c>
     </row>
@@ -997,7 +997,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 11. Миграция</t>
+          <t xml:space="preserve">Миграция</t>
         </is>
       </c>
       <c r="D33" s="6">
@@ -1005,12 +1005,12 @@
       </c>
       <c r="E33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты переносят учебную базу на новую версию схемы с сохранением данных. Сдают скрипты миграции и отката и отчёт о проверке данных.</t>
+          <t xml:space="preserve">Меняют схему MySQL через ALTER TABLE, заполняют новое поле и проверяют обратный скрипт. Сдают миграцию и откат.</t>
         </is>
       </c>
       <c r="F33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">версия схемы, откат, перенос данных, проверка, скрипт, совместимость</t>
+          <t xml:space="preserve">ALTER TABLE, schema_version, backfill, rollback, миграция, проверка</t>
         </is>
       </c>
     </row>
@@ -1027,7 +1027,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Практика 12. Итоговая БД</t>
+          <t xml:space="preserve">Итоговая база и .NET-приложение</t>
         </is>
       </c>
       <c r="D34" s="6">
@@ -1035,12 +1035,12 @@
       </c>
       <c r="E34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Студенты собирают учебную базу целиком: схема, роли, индексы, копия и скрипт обслуживания. Сдают базу и комплект скриптов с протоколом проверки.</t>
+          <t xml:space="preserve">Собирают итоговую базу MySQL и .NET-приложение: схема, роли, индексы, дамп, обслуживание. Сдают комплект и протокол.</t>
         </is>
       </c>
       <c r="F34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">схема, ограничение, роль, индекс, копия, чек-лист</t>
+          <t xml:space="preserve">MySQL, схема, роль, индекс, дамп, .NET</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add all is-design lessons and finish the site-wide polish
Renames references to spo-it-materials, restores lecture and practice prefixes in the database automation plan, sorts discipline cards by availability and subject number, and shows draw.io without the browser label. All 50 is-design lessons are written with 26 lectures and 24 practices. Discipline cards keep the lesson count and exam or credit without the СПО label or hours.
</commit_message>
<xml_diff>
--- a/courses/4/db-automation/dist/Учебный_план_Управление_и_автоматизация_баз_данных.xlsx
+++ b/courses/4/db-automation/dist/Учебный_план_Управление_и_автоматизация_баз_данных.xlsx
@@ -187,7 +187,7 @@
       </c>
       <c r="C6" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Управление и автоматизация БД</t>
+          <t xml:space="preserve">Лекция 1. Управление и автоматизация БД</t>
         </is>
       </c>
       <c r="D6" s="6">
@@ -217,7 +217,7 @@
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Архитектура MySQL и InnoDB</t>
+          <t xml:space="preserve">Лекция 2. Архитектура MySQL и InnoDB</t>
         </is>
       </c>
       <c r="D7" s="6">
@@ -247,7 +247,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">XAMPP, MySQL и подключение из .NET</t>
+          <t xml:space="preserve">Лекция 3. XAMPP, MySQL и подключение из .NET</t>
         </is>
       </c>
       <c r="D8" s="6">
@@ -277,7 +277,7 @@
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Запуск XAMPP, база utf8mb4, подключение из .NET</t>
+          <t xml:space="preserve">Практика 1. Запуск XAMPP, база utf8mb4, подключение из .NET</t>
         </is>
       </c>
       <c r="D9" s="6">
@@ -307,7 +307,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Пользователи и роли MySQL</t>
+          <t xml:space="preserve">Лекция 4. Пользователи и роли MySQL</t>
         </is>
       </c>
       <c r="D10" s="6">
@@ -337,7 +337,7 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Роли и доступ в MySQL</t>
+          <t xml:space="preserve">Практика 2. Роли и доступ в MySQL</t>
         </is>
       </c>
       <c r="D11" s="6">
@@ -367,7 +367,7 @@
       </c>
       <c r="C12" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Резервное копирование MySQL</t>
+          <t xml:space="preserve">Лекция 5. Резервное копирование MySQL</t>
         </is>
       </c>
       <c r="D12" s="6">
@@ -397,7 +397,7 @@
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Восстановление и журналы MySQL</t>
+          <t xml:space="preserve">Лекция 6. Восстановление и журналы MySQL</t>
         </is>
       </c>
       <c r="D13" s="6">
@@ -427,7 +427,7 @@
       </c>
       <c r="C14" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Резервное копирование и восстановление</t>
+          <t xml:space="preserve">Практика 3. Резервное копирование и восстановление</t>
         </is>
       </c>
       <c r="D14" s="6">
@@ -457,7 +457,7 @@
       </c>
       <c r="C15" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Репликация MySQL</t>
+          <t xml:space="preserve">Лекция 7. Репликация MySQL</t>
         </is>
       </c>
       <c r="D15" s="6">
@@ -487,7 +487,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Индексы и производительность InnoDB</t>
+          <t xml:space="preserve">Лекция 8. Индексы и производительность InnoDB</t>
         </is>
       </c>
       <c r="D16" s="6">
@@ -517,7 +517,7 @@
       </c>
       <c r="C17" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Оптимизация запросов MySQL</t>
+          <t xml:space="preserve">Лекция 9. Оптимизация запросов MySQL</t>
         </is>
       </c>
       <c r="D17" s="6">
@@ -547,7 +547,7 @@
       </c>
       <c r="C18" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Индексы и оптимизация</t>
+          <t xml:space="preserve">Практика 4. Индексы и оптимизация</t>
         </is>
       </c>
       <c r="D18" s="6">
@@ -577,7 +577,7 @@
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Транзакции и блокировки InnoDB</t>
+          <t xml:space="preserve">Лекция 10. Транзакции и блокировки InnoDB</t>
         </is>
       </c>
       <c r="D19" s="6">
@@ -607,7 +607,7 @@
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Транзакции</t>
+          <t xml:space="preserve">Практика 5. Транзакции</t>
         </is>
       </c>
       <c r="D20" s="6">
@@ -637,7 +637,7 @@
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Импорт и экспорт данных</t>
+          <t xml:space="preserve">Лекция 11. Импорт и экспорт данных</t>
         </is>
       </c>
       <c r="D21" s="6">
@@ -667,7 +667,7 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Импорт JSON</t>
+          <t xml:space="preserve">Практика 6. Импорт JSON</t>
         </is>
       </c>
       <c r="D22" s="6">
@@ -697,7 +697,7 @@
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Экспорт</t>
+          <t xml:space="preserve">Практика 7. Экспорт</t>
         </is>
       </c>
       <c r="D23" s="6">
@@ -727,7 +727,7 @@
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Автоматизация на C# и .NET SDK 10</t>
+          <t xml:space="preserve">Лекция 12. Автоматизация на C# и .NET SDK 10</t>
         </is>
       </c>
       <c r="D24" s="6">
@@ -757,7 +757,7 @@
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Консольное приложение обслуживания</t>
+          <t xml:space="preserve">Практика 8. Консольное приложение обслуживания</t>
         </is>
       </c>
       <c r="D25" s="6">
@@ -787,7 +787,7 @@
       </c>
       <c r="C26" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Планировщик заданий и события MySQL</t>
+          <t xml:space="preserve">Лекция 13. Планировщик заданий и события MySQL</t>
         </is>
       </c>
       <c r="D26" s="6">
@@ -817,7 +817,7 @@
       </c>
       <c r="C27" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Мониторинг MySQL и приложение WinForms</t>
+          <t xml:space="preserve">Лекция 14. Мониторинг MySQL и приложение WinForms</t>
         </is>
       </c>
       <c r="D27" s="6">
@@ -847,7 +847,7 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Планировщик и мониторинг</t>
+          <t xml:space="preserve">Практика 9. Планировщик и мониторинг</t>
         </is>
       </c>
       <c r="D28" s="6">
@@ -877,7 +877,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аудит MySQL</t>
+          <t xml:space="preserve">Лекция 15. Аудит MySQL</t>
         </is>
       </c>
       <c r="D29" s="6">
@@ -907,7 +907,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Безопасность MySQL и .NET</t>
+          <t xml:space="preserve">Лекция 16. Безопасность MySQL и .NET</t>
         </is>
       </c>
       <c r="D30" s="6">
@@ -937,7 +937,7 @@
       </c>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Аудит и безопасность</t>
+          <t xml:space="preserve">Практика 10. Аудит и безопасность</t>
         </is>
       </c>
       <c r="D31" s="6">
@@ -967,7 +967,7 @@
       </c>
       <c r="C32" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Миграции схемы MySQL</t>
+          <t xml:space="preserve">Лекция 17. Миграции схемы MySQL</t>
         </is>
       </c>
       <c r="D32" s="6">
@@ -997,7 +997,7 @@
       </c>
       <c r="C33" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Миграция</t>
+          <t xml:space="preserve">Практика 11. Миграция</t>
         </is>
       </c>
       <c r="D33" s="6">
@@ -1027,7 +1027,7 @@
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">Итоговая база и .NET-приложение</t>
+          <t xml:space="preserve">Практика 12. Итоговая база и .NET-приложение</t>
         </is>
       </c>
       <c r="D34" s="6">

</xml_diff>